<commit_message>
instagram profile posts, added orizaba tasks, video features extractor
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscarcuellar/ocn/media/apify_client/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C35EEDF9-A5AB-6C4A-A46F-54C56012853B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC2A3963-7041-724A-B3A5-6646F1844035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1560" windowWidth="19420" windowHeight="20780" xr2:uid="{52EE6F4F-3953-A140-B2A6-0482DE438E94}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="31920" windowHeight="20780" xr2:uid="{52EE6F4F-3953-A140-B2A6-0482DE438E94}"/>
   </bookViews>
   <sheets>
     <sheet name="tasks" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="61">
   <si>
     <t>task_id</t>
   </si>
@@ -138,6 +138,84 @@
   </si>
   <si>
     <t>https://www.facebook.com/poderciudadanoradio</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/ChismeOrizabaMx</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/1233543673337523/</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>Balaceras Orizaba 2</t>
+  </si>
+  <si>
+    <t>Chisme Orizabeño</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/unpocodeorizabaa</t>
+  </si>
+  <si>
+    <t>GROUPS</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/386982481787894</t>
+  </si>
+  <si>
+    <t>balaceras y noticias sin censura “orizaba y zona centro de Veracruz”</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/profile.php?id=61586769881432</t>
+  </si>
+  <si>
+    <t>Notimendez</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/ORIZABA.PROYECTOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orizaba Proyectos </t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/OrizabaCapital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orizaba Capital </t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/groups/enterateorizaba</t>
+  </si>
+  <si>
+    <t>Entérate Orizaba</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/OrizabaVer</t>
+  </si>
+  <si>
+    <t>El Vigilante Orizabeño</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/www.orizabaenred.com.mx</t>
+  </si>
+  <si>
+    <t>Orizaba en Red</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/elbuentonodecordoba</t>
+  </si>
+  <si>
+    <t>El buen tono de cordoba</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/ElMundodeOrizaba</t>
+  </si>
+  <si>
+    <t>El Mundo de Orizaba</t>
+  </si>
+  <si>
+    <t>Un Poco de Orizava</t>
   </si>
 </sst>
 </file>
@@ -1009,14 +1087,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CF29DF0-388E-0142-B0F1-7C2350E3D19C}">
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:S22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="19.6640625" customWidth="1"/>
-    <col min="3" max="3" width="36.1640625" customWidth="1"/>
+    <col min="2" max="3" width="19.6640625" customWidth="1"/>
+    <col min="4" max="4" width="36.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1024,370 +1102,824 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>19</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>20</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>21</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>22</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>30</v>
       </c>
-      <c r="I2" t="b">
-        <v>0</v>
-      </c>
       <c r="J2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+      <c r="S2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>24</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>19</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>21</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>25</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>50</v>
       </c>
-      <c r="I3" t="b">
-        <v>0</v>
-      </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" t="b">
-        <v>0</v>
-      </c>
-      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="L3" t="b">
+        <v>0</v>
+      </c>
+      <c r="M3">
         <v>15</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>30</v>
       </c>
-      <c r="P3" t="b">
-        <v>1</v>
-      </c>
       <c r="Q3" t="b">
-        <v>0</v>
-      </c>
-      <c r="R3" t="s">
+        <v>1</v>
+      </c>
+      <c r="R3" t="b">
+        <v>0</v>
+      </c>
+      <c r="S3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>20</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>21</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>25</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>50</v>
       </c>
-      <c r="I4" t="b">
-        <v>0</v>
-      </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="b">
-        <v>0</v>
-      </c>
-      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4">
         <v>15</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>30</v>
       </c>
-      <c r="P4" t="b">
-        <v>1</v>
-      </c>
       <c r="Q4" t="b">
-        <v>0</v>
-      </c>
-      <c r="R4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>20</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>21</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>25</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>30</v>
       </c>
-      <c r="I5" t="b">
-        <v>1</v>
-      </c>
       <c r="J5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="b">
-        <v>1</v>
-      </c>
-      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5">
         <v>15</v>
       </c>
-      <c r="P5" t="b">
-        <v>0</v>
-      </c>
       <c r="Q5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="R5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>28</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>31</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>25</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>30</v>
       </c>
-      <c r="I6" t="b">
-        <v>1</v>
-      </c>
       <c r="J6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="b">
-        <v>1</v>
-      </c>
-      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6">
         <v>15</v>
       </c>
-      <c r="P6" t="b">
-        <v>0</v>
-      </c>
       <c r="Q6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="R6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>28</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>32</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>25</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>30</v>
       </c>
-      <c r="I7" t="b">
-        <v>1</v>
-      </c>
       <c r="J7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K7" t="b">
-        <v>1</v>
-      </c>
-      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7">
         <v>15</v>
       </c>
-      <c r="P7" t="b">
-        <v>0</v>
-      </c>
       <c r="Q7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="R7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>25</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>50</v>
       </c>
-      <c r="I8" t="b">
-        <v>1</v>
-      </c>
       <c r="J8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" t="b">
-        <v>1</v>
-      </c>
-      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="M8">
         <v>15</v>
       </c>
-      <c r="P8" t="b">
-        <v>0</v>
-      </c>
       <c r="Q8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="R8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>25</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>50</v>
       </c>
-      <c r="I9" t="b">
-        <v>1</v>
-      </c>
       <c r="J9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="M9">
         <v>15</v>
       </c>
-      <c r="P9" t="b">
-        <v>0</v>
-      </c>
       <c r="Q9" t="b">
+        <v>0</v>
+      </c>
+      <c r="R9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" t="s">
+        <v>25</v>
+      </c>
+      <c r="I10">
+        <v>20</v>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10">
+        <v>10</v>
+      </c>
+      <c r="Q10" t="b">
+        <v>0</v>
+      </c>
+      <c r="R10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" t="s">
+        <v>44</v>
+      </c>
+      <c r="H11" t="s">
+        <v>25</v>
+      </c>
+      <c r="I11">
+        <v>20</v>
+      </c>
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11">
+        <v>10</v>
+      </c>
+      <c r="Q11" t="b">
+        <v>0</v>
+      </c>
+      <c r="R11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" t="s">
+        <v>46</v>
+      </c>
+      <c r="H12" t="s">
+        <v>25</v>
+      </c>
+      <c r="I12">
+        <v>10</v>
+      </c>
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12">
+        <v>10</v>
+      </c>
+      <c r="Q12" t="b">
+        <v>0</v>
+      </c>
+      <c r="R12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" t="s">
+        <v>48</v>
+      </c>
+      <c r="H13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I13">
+        <v>5</v>
+      </c>
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K13" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+      <c r="M13">
+        <v>10</v>
+      </c>
+      <c r="Q13" t="b">
+        <v>0</v>
+      </c>
+      <c r="R13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" t="s">
+        <v>52</v>
+      </c>
+      <c r="H14" t="s">
+        <v>25</v>
+      </c>
+      <c r="I14">
+        <v>20</v>
+      </c>
+      <c r="J14" t="b">
+        <v>1</v>
+      </c>
+      <c r="K14" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+      <c r="M14">
+        <v>10</v>
+      </c>
+      <c r="Q14" t="b">
+        <v>0</v>
+      </c>
+      <c r="R14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" t="s">
+        <v>54</v>
+      </c>
+      <c r="H15" t="s">
+        <v>25</v>
+      </c>
+      <c r="I15">
+        <v>30</v>
+      </c>
+      <c r="J15" t="b">
+        <v>1</v>
+      </c>
+      <c r="K15" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+      <c r="M15">
+        <v>20</v>
+      </c>
+      <c r="Q15" t="b">
+        <v>0</v>
+      </c>
+      <c r="R15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" t="s">
+        <v>56</v>
+      </c>
+      <c r="H16" t="s">
+        <v>25</v>
+      </c>
+      <c r="I16">
+        <v>50</v>
+      </c>
+      <c r="J16" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>20</v>
+      </c>
+      <c r="Q16" t="b">
+        <v>0</v>
+      </c>
+      <c r="R16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" t="s">
+        <v>58</v>
+      </c>
+      <c r="H17" t="s">
+        <v>25</v>
+      </c>
+      <c r="I17">
+        <v>25</v>
+      </c>
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+      <c r="K17" t="b">
+        <v>1</v>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+      <c r="M17">
+        <v>15</v>
+      </c>
+      <c r="Q17" t="b">
+        <v>0</v>
+      </c>
+      <c r="R17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H18" t="s">
+        <v>25</v>
+      </c>
+      <c r="I18">
+        <v>35</v>
+      </c>
+      <c r="J18" t="b">
+        <v>0</v>
+      </c>
+      <c r="K18" t="b">
+        <v>1</v>
+      </c>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>15</v>
+      </c>
+      <c r="Q18" t="b">
+        <v>0</v>
+      </c>
+      <c r="R18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D19" t="s">
+        <v>40</v>
+      </c>
+      <c r="H19" t="s">
+        <v>25</v>
+      </c>
+      <c r="I19">
+        <v>30</v>
+      </c>
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+      <c r="K19" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+      <c r="M19">
+        <v>5</v>
+      </c>
+      <c r="Q19" t="b">
+        <v>0</v>
+      </c>
+      <c r="R19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" t="s">
+        <v>38</v>
+      </c>
+      <c r="D20" t="s">
+        <v>36</v>
+      </c>
+      <c r="H20" t="s">
+        <v>25</v>
+      </c>
+      <c r="J20" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="b">
+        <v>0</v>
+      </c>
+      <c r="R20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" t="s">
+        <v>42</v>
+      </c>
+      <c r="H21" t="s">
+        <v>25</v>
+      </c>
+      <c r="J21" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="b">
+        <v>0</v>
+      </c>
+      <c r="R21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="J22" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="b">
+        <v>0</v>
+      </c>
+      <c r="R22" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C5" r:id="rId1" xr:uid="{84C75881-B9D2-E44E-8630-7B96894C43D7}"/>
-    <hyperlink ref="C9" r:id="rId2" xr:uid="{B90AFFFE-004B-9A40-B82B-C98A3D5105AF}"/>
-    <hyperlink ref="C8" r:id="rId3" xr:uid="{EC5B7B07-DA9A-E84A-8B02-2C6AF7BC807D}"/>
+    <hyperlink ref="D5" r:id="rId1" xr:uid="{84C75881-B9D2-E44E-8630-7B96894C43D7}"/>
+    <hyperlink ref="D9" r:id="rId2" xr:uid="{B90AFFFE-004B-9A40-B82B-C98A3D5105AF}"/>
+    <hyperlink ref="D8" r:id="rId3" xr:uid="{EC5B7B07-DA9A-E84A-8B02-2C6AF7BC807D}"/>
+    <hyperlink ref="D18" r:id="rId4" xr:uid="{DD330F28-7ADD-0746-A7C6-E2C6EE4C83DB}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add date/post date to attached news, enrich author to fb keyword search, raise rabbit exceptions
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscarcuellar/ocn/media/apify_client/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C123BBC-C9DD-BE41-9402-E65AF901FCB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8681C6-971E-3E42-AA81-D6DE234F5BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="31920" windowHeight="20780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="38980" windowHeight="26620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tasks" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="167">
   <si>
     <t>task_id</t>
   </si>
@@ -903,7 +903,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U83"/>
+  <dimension ref="A1:U84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="4" width="19.6640625" customWidth="1"/>
@@ -1140,7 +1140,7 @@
         <v>26</v>
       </c>
       <c r="K5">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="L5" t="b">
         <v>1</v>
@@ -1184,7 +1184,7 @@
         <v>26</v>
       </c>
       <c r="K6">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="L6" t="b">
         <v>1</v>
@@ -4914,6 +4914,47 @@
         <v>0</v>
       </c>
       <c r="T83" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A84">
+        <v>84</v>
+      </c>
+      <c r="B84" t="s">
+        <v>100</v>
+      </c>
+      <c r="C84" t="s">
+        <v>150</v>
+      </c>
+      <c r="D84" t="s">
+        <v>150</v>
+      </c>
+      <c r="E84" t="s">
+        <v>150</v>
+      </c>
+      <c r="J84" t="s">
+        <v>26</v>
+      </c>
+      <c r="K84">
+        <v>5</v>
+      </c>
+      <c r="L84" t="b">
+        <v>1</v>
+      </c>
+      <c r="M84" t="b">
+        <v>1</v>
+      </c>
+      <c r="N84" t="b">
+        <v>1</v>
+      </c>
+      <c r="O84">
+        <v>15</v>
+      </c>
+      <c r="S84" t="b">
+        <v>1</v>
+      </c>
+      <c r="T84" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
facebook keyword search cleanu
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscarcuellar/ocn/media/apify_client/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8681C6-971E-3E42-AA81-D6DE234F5BFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5C6E10D-FB04-1447-88D5-598FA7FF75D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="38980" windowHeight="26620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="169">
   <si>
     <t>task_id</t>
   </si>
@@ -521,6 +521,12 @@
   </si>
   <si>
     <t>FeliFer Macías</t>
+  </si>
+  <si>
+    <t>{"get_comments_after_likes": 100, "enrich_author_after_likes": 100}</t>
+  </si>
+  <si>
+    <t>Conserva sólo las publicaciones que hablen de eventos o temas de interés común en el estado o ciudad de Querétaro (en general, temas que puedan ser de interés para el gobierno, ejemplo no exhaustivo: Emergencias, infraestructura, eventos culturales, servicios públicos, seguridad, ... entre otros). Elimina las preguntas de usuarios, ofertas de ventas, saludos, etc,)</t>
   </si>
 </sst>
 </file>
@@ -4785,7 +4791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>81</v>
       </c>
@@ -4829,7 +4835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>82</v>
       </c>
@@ -4873,7 +4879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>83</v>
       </c>
@@ -4917,7 +4923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>84</v>
       </c>
@@ -4937,7 +4943,7 @@
         <v>26</v>
       </c>
       <c r="K84">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="L84" t="b">
         <v>1</v>
@@ -4951,11 +4957,17 @@
       <c r="O84">
         <v>15</v>
       </c>
+      <c r="Q84" t="s">
+        <v>168</v>
+      </c>
       <c r="S84" t="b">
         <v>1</v>
       </c>
       <c r="T84" t="b">
         <v>1</v>
+      </c>
+      <c r="U84" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add update_existing param, log filtered documents
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscarcuellar/ocn/media/apify_client/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EFA1D13-B1B2-334F-984E-A99A98EF73A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA315F9B-B1C7-4B49-B3FC-FDC8052D3668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="31920" windowHeight="20780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6680" yWindow="700" windowWidth="38980" windowHeight="26620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tasks" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="713" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="181">
   <si>
     <t>task_id</t>
   </si>
@@ -564,6 +564,18 @@
   </si>
   <si>
     <t>zona fest</t>
+  </si>
+  <si>
+    <t>Conserva sólo las publicaciones que hablen del evento Zona Fest en Querétaro, o temas relacionados</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>{"timeframe":"7d","enrich":true}</t>
+  </si>
+  <si>
+    <t>update_existing</t>
   </si>
 </sst>
 </file>
@@ -946,7 +958,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U87"/>
+  <dimension ref="A1:V88"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="4" width="19.6640625" customWidth="1"/>
@@ -954,7 +966,7 @@
     <col min="6" max="6" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1018,8 +1030,11 @@
       <c r="U1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1054,7 +1069,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1104,7 +1119,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1154,7 +1169,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1204,7 +1219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1248,7 +1263,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1292,7 +1307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1336,7 +1351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1380,7 +1395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1421,7 +1436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1462,7 +1477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1503,7 +1518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1544,7 +1559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1585,7 +1600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1626,7 +1641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -4828,7 +4843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>81</v>
       </c>
@@ -4872,7 +4887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>82</v>
       </c>
@@ -4916,7 +4931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>83</v>
       </c>
@@ -4960,7 +4975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>84</v>
       </c>
@@ -5007,7 +5022,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="85" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>85</v>
       </c>
@@ -5054,7 +5069,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="86" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>86</v>
       </c>
@@ -5101,9 +5116,9 @@
         <v>167</v>
       </c>
     </row>
-    <row r="87" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A87">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B87" t="s">
         <v>100</v>
@@ -5133,10 +5148,10 @@
         <v>1</v>
       </c>
       <c r="O87">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="Q87" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="S87" t="b">
         <v>1</v>
@@ -5146,6 +5161,50 @@
       </c>
       <c r="U87" t="s">
         <v>167</v>
+      </c>
+      <c r="V87" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <v>88</v>
+      </c>
+      <c r="B88" t="s">
+        <v>19</v>
+      </c>
+      <c r="C88" t="s">
+        <v>150</v>
+      </c>
+      <c r="D88" t="s">
+        <v>175</v>
+      </c>
+      <c r="E88" t="s">
+        <v>175</v>
+      </c>
+      <c r="G88" t="s">
+        <v>21</v>
+      </c>
+      <c r="H88" t="s">
+        <v>22</v>
+      </c>
+      <c r="J88" t="s">
+        <v>178</v>
+      </c>
+      <c r="K88">
+        <v>50</v>
+      </c>
+      <c r="L88" t="b">
+        <v>1</v>
+      </c>
+      <c r="M88" t="b">
+        <v>1</v>
+      </c>
+      <c r="N88" t="b">
+        <v>0</v>
+      </c>
+      <c r="U88" t="s">
+        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
parsed tiktok comments from apify dataset id
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscarcuellar/ocn/media/apify_client/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2DEF5D-F99A-2949-AF75-909CB3812875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85B0D6EC-1CB1-484D-B240-0B00C83F9422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6680" yWindow="700" windowWidth="32860" windowHeight="26620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="184">
   <si>
     <t>task_id</t>
   </si>
@@ -576,6 +576,15 @@
   </si>
   <si>
     <t>update_existing</t>
+  </si>
+  <si>
+    <t>mexicozonafest</t>
+  </si>
+  <si>
+    <t>zonafest</t>
+  </si>
+  <si>
+    <t>tiktok_posts</t>
   </si>
 </sst>
 </file>
@@ -958,7 +967,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V88"/>
+  <dimension ref="A1:V91"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="4" width="19.6640625" customWidth="1"/>
@@ -5205,6 +5214,153 @@
       </c>
       <c r="U88" t="s">
         <v>179</v>
+      </c>
+    </row>
+    <row r="89" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <v>89</v>
+      </c>
+      <c r="B89" t="s">
+        <v>100</v>
+      </c>
+      <c r="C89" t="s">
+        <v>150</v>
+      </c>
+      <c r="D89" t="s">
+        <v>175</v>
+      </c>
+      <c r="E89" t="s">
+        <v>181</v>
+      </c>
+      <c r="J89" t="s">
+        <v>26</v>
+      </c>
+      <c r="K89">
+        <v>100</v>
+      </c>
+      <c r="L89" t="b">
+        <v>1</v>
+      </c>
+      <c r="M89" t="b">
+        <v>1</v>
+      </c>
+      <c r="N89" t="b">
+        <v>1</v>
+      </c>
+      <c r="O89">
+        <v>25</v>
+      </c>
+      <c r="Q89" t="s">
+        <v>177</v>
+      </c>
+      <c r="S89" t="b">
+        <v>1</v>
+      </c>
+      <c r="T89" t="b">
+        <v>1</v>
+      </c>
+      <c r="U89" t="s">
+        <v>167</v>
+      </c>
+      <c r="V89" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <v>90</v>
+      </c>
+      <c r="B90" t="s">
+        <v>100</v>
+      </c>
+      <c r="C90" t="s">
+        <v>150</v>
+      </c>
+      <c r="D90" t="s">
+        <v>175</v>
+      </c>
+      <c r="E90" t="s">
+        <v>182</v>
+      </c>
+      <c r="J90" t="s">
+        <v>26</v>
+      </c>
+      <c r="K90">
+        <v>100</v>
+      </c>
+      <c r="L90" t="b">
+        <v>1</v>
+      </c>
+      <c r="M90" t="b">
+        <v>1</v>
+      </c>
+      <c r="N90" t="b">
+        <v>1</v>
+      </c>
+      <c r="O90">
+        <v>25</v>
+      </c>
+      <c r="Q90" t="s">
+        <v>177</v>
+      </c>
+      <c r="S90" t="b">
+        <v>1</v>
+      </c>
+      <c r="T90" t="b">
+        <v>1</v>
+      </c>
+      <c r="U90" t="s">
+        <v>167</v>
+      </c>
+      <c r="V90" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <v>91</v>
+      </c>
+      <c r="B91" t="s">
+        <v>183</v>
+      </c>
+      <c r="C91" t="s">
+        <v>150</v>
+      </c>
+      <c r="D91" t="s">
+        <v>175</v>
+      </c>
+      <c r="E91" t="s">
+        <v>182</v>
+      </c>
+      <c r="J91" t="s">
+        <v>26</v>
+      </c>
+      <c r="K91">
+        <v>100</v>
+      </c>
+      <c r="L91" t="b">
+        <v>1</v>
+      </c>
+      <c r="M91" t="b">
+        <v>1</v>
+      </c>
+      <c r="N91" t="b">
+        <v>1</v>
+      </c>
+      <c r="O91">
+        <v>25</v>
+      </c>
+      <c r="Q91" t="s">
+        <v>177</v>
+      </c>
+      <c r="S91" t="b">
+        <v>1</v>
+      </c>
+      <c r="T91" t="b">
+        <v>1</v>
+      </c>
+      <c r="V91" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added safe mongo fallback when not reachable, topics parameter to google news
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscarcuellar/ocn/media/apify_client/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85B0D6EC-1CB1-484D-B240-0B00C83F9422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCBD7FA6-8465-AF4D-8B6D-FBC8E318AD79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6680" yWindow="700" windowWidth="32860" windowHeight="26620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="185">
   <si>
     <t>task_id</t>
   </si>
@@ -585,6 +585,9 @@
   </si>
   <si>
     <t>tiktok_posts</t>
+  </si>
+  <si>
+    <t>Conserva sólo las publicaciones que hablen del evento Zona Fest en Querétaro, o temas relacionados (si menciona Zona Fest o variaciones y parece ser de México es muy probable que sí se refiera a este evento)</t>
   </si>
 </sst>
 </file>
@@ -5332,11 +5335,14 @@
       <c r="E91" t="s">
         <v>182</v>
       </c>
+      <c r="G91" t="s">
+        <v>21</v>
+      </c>
       <c r="J91" t="s">
-        <v>26</v>
+        <v>178</v>
       </c>
       <c r="K91">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="L91" t="b">
         <v>1</v>
@@ -5351,7 +5357,7 @@
         <v>25</v>
       </c>
       <c r="Q91" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="S91" t="b">
         <v>1</v>

</xml_diff>